<commit_message>
Fine Dining Checklists Kit Pro (EN): remontaje tras la ronda de revisión final y republicación en dl/ (VPS)
Montaje idempotente; gates VERDE 8/0; autotest 19/19; censo-entregables 0, no-latinos 0, LIT255 verde; volcado EN regenerado.

Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/fine-dining-checklist-templates/02-tasting-menu-mise-en-place-checklist.xlsx
+++ b/astro-site/public/dl/fine-dining-checklist-templates/02-tasting-menu-mise-en-place-checklist.xlsx
@@ -1104,7 +1104,7 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Long sous vide: meat cuts (48–72 hr at low temp.). Cook to the time and temperature of your validated recipe; if chilled and stored in the bag (reduced oxygen packaging), you need a HACCP plan or health department variance (FDA Food Code 3-502.11 / 3-502.12); chill from 135 °F to 70 °F within 2 hr and to 41 °F within 4 more hr (3-501.14)</t>
+          <t>Long sous vide: meat cuts (48–72 hr at low temp.). Cook to the time and temperature of your validated recipe (FDA Food Code 3-401.11 time/temperature tables); if chilled and stored in the bag (reduced oxygen packaging), you need a HACCP plan or health department variance (FDA Food Code 3-502.11 / 3-502.12); chill from 135 °F to 70 °F within 2 hr and to 41 °F within 4 more hr (3-501.14)</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Mid-lead sous vide: fish and shellfish (6–12 hr)</t>
+          <t>Mid-lead sous vide: fish and shellfish (6–12 hr); if bagged and chilled or held (reduced oxygen packaging), a HACCP plan or health department variance (FDA Food Code 3-502.11 / 3-502.12); chill per 3-501.14</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Slow confits (duck, pork, octopus)</t>
+          <t>Slow confits (duck, pork, octopus); if bagged and chilled, the same HACCP plan or variance (FDA Food Code 3-502.11 / 3-502.12); chill per 3-501.14</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">

</xml_diff>